<commit_message>
Finalize Track A/B interleaving and empirical run closure artifacts
</commit_message>
<xml_diff>
--- a/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/cf_wave1/SCN-EB033-CF-TABLE-SPILL.xlsx
+++ b/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/cf_wave1/SCN-EB033-CF-TABLE-SPILL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\DnaCalc\Foundation\research\runs\20260228-180047-excel-compat-empirical-pass-01\fixtures\cf_wave1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC9B5145-30B7-47C5-8886-571295178BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93CE74D7-CDF4-43D1-BBE3-D6F55D24E3E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7440" yWindow="3075" windowWidth="17460" windowHeight="11595" xr2:uid="{F4EC6ACB-7F94-4838-A308-D94877A653F8}"/>
+    <workbookView xWindow="3135" yWindow="3885" windowWidth="11955" windowHeight="11595" xr2:uid="{074F1F70-0A4C-477F-9B25-DD5D0D0D3F1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -121,11 +121,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D873DFF4-D3B9-4482-8FAC-A4D920C56874}" name="TblCfWave1" displayName="TblCfWave1" ref="A1:B3" totalsRowShown="0">
-  <autoFilter ref="A1:B3" xr:uid="{D873DFF4-D3B9-4482-8FAC-A4D920C56874}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7D253A1B-CA4B-42AD-B1C1-BEA474DA1B4D}" name="TblCfWave1" displayName="TblCfWave1" ref="A1:B3" totalsRowShown="0">
+  <autoFilter ref="A1:B3" xr:uid="{7D253A1B-CA4B-42AD-B1C1-BEA474DA1B4D}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{562D027D-BD9B-4A35-B520-4A816F35BC61}" name="Name"/>
-    <tableColumn id="2" xr3:uid="{3DA449FD-C49E-4AC1-A8CA-6FBF7800C4CD}" name="Val"/>
+    <tableColumn id="1" xr3:uid="{60CC03FE-D8CB-46FA-A076-A69B03246DBC}" name="Name"/>
+    <tableColumn id="2" xr3:uid="{9A2BC6AB-03F1-4371-B18B-7EAB18B50747}" name="Val"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -447,7 +447,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DA0BB1-A287-4C2D-BE0C-08FA8330E053}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C8F8E32-1C91-4D4F-99B1-B7ED7D6865D9}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>